<commit_message>
Added rates per unit information to resource usage baseline tab
</commit_message>
<xml_diff>
--- a/Documentation/Management/Reports/FlyDreamAir_Most_Valuable_Resource.xlsx
+++ b/Documentation/Management/Reports/FlyDreamAir_Most_Valuable_Resource.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UOW\CSIT214 IT Project Management\FlyDreamAir\docs\management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UOW\CSIT214 IT Project Management\FlyDreamAir\Documentation\Management\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B97A1CD6-3512-42B5-9658-4AAED8015E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73658B7-8EA9-4D6C-A238-764A529B9672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{64F56E0A-39E6-49DC-9E83-6C856E3BAFBB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{64F56E0A-39E6-49DC-9E83-6C856E3BAFBB}"/>
   </bookViews>
   <sheets>
     <sheet name="Resourse Usage Baseline" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="Financial Analysis" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="253">
   <si>
     <t>Human</t>
   </si>
@@ -788,6 +787,18 @@
   </si>
   <si>
     <t>Note: Add Actuals once project completed.</t>
+  </si>
+  <si>
+    <t>Hour</t>
+  </si>
+  <si>
+    <t>Each</t>
+  </si>
+  <si>
+    <t>Yearly</t>
+  </si>
+  <si>
+    <t>Rates</t>
   </si>
 </sst>
 </file>
@@ -844,7 +855,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -884,6 +895,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -983,7 +1000,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1045,20 +1062,14 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="8" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1066,6 +1077,17 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1410,6 +1432,7 @@
     <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1428,6 +1451,12 @@
       <c r="E1" s="2" t="s">
         <v>46</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
@@ -1439,7 +1468,7 @@
         <f>SUM(D3,D11,D22,D30,D49)</f>
         <v>792</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="56">
         <f>SUM(E3,E11,E22,E30,E49)</f>
         <v>65640</v>
       </c>
@@ -1454,9 +1483,15 @@
         <f>SUM(D4:D10)</f>
         <v>96</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="57">
         <f>SUM(E4:E10)</f>
         <v>8160</v>
+      </c>
+      <c r="F3" s="59">
+        <v>85</v>
+      </c>
+      <c r="G3" s="60" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1470,7 +1505,7 @@
       <c r="D4" s="10">
         <v>40</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="58">
         <v>3400</v>
       </c>
     </row>
@@ -1485,7 +1520,7 @@
       <c r="D5" s="10">
         <v>8</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="58">
         <v>680</v>
       </c>
     </row>
@@ -1500,7 +1535,7 @@
       <c r="D6" s="10">
         <v>4</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="58">
         <v>340</v>
       </c>
     </row>
@@ -1515,7 +1550,7 @@
       <c r="D7" s="10">
         <v>24</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="58">
         <v>2040</v>
       </c>
     </row>
@@ -1530,16 +1565,16 @@
       <c r="D8" s="10">
         <v>8</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="58">
         <v>680</v>
       </c>
-      <c r="I8" s="53" t="s">
+      <c r="I8" s="50" t="s">
         <v>248</v>
       </c>
-      <c r="J8" s="53"/>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
+      <c r="J8" s="50"/>
+      <c r="K8" s="50"/>
+      <c r="L8" s="50"/>
+      <c r="M8" s="50"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
@@ -1552,14 +1587,14 @@
       <c r="D9" s="10">
         <v>4</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="58">
         <v>340</v>
       </c>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
-      <c r="M9" s="53"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
@@ -1572,14 +1607,14 @@
       <c r="D10" s="10">
         <v>8</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="58">
         <v>680</v>
       </c>
-      <c r="I10" s="53"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
-      <c r="M10" s="53"/>
+      <c r="I10" s="50"/>
+      <c r="J10" s="50"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
@@ -1591,9 +1626,15 @@
         <f>SUM(D12:D21)</f>
         <v>152</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="57">
         <f>SUM(E12:E21)</f>
         <v>11400</v>
+      </c>
+      <c r="F11" s="59">
+        <v>75</v>
+      </c>
+      <c r="G11" s="60" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -1607,7 +1648,7 @@
       <c r="D12" s="10">
         <v>40</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="58">
         <v>3000</v>
       </c>
     </row>
@@ -1622,7 +1663,7 @@
       <c r="D13" s="10">
         <v>16</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="58">
         <v>1200</v>
       </c>
     </row>
@@ -1637,7 +1678,7 @@
       <c r="D14" s="10">
         <v>16</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="58">
         <v>1200</v>
       </c>
     </row>
@@ -1652,7 +1693,7 @@
       <c r="D15" s="10">
         <v>20</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="58">
         <v>1500</v>
       </c>
     </row>
@@ -1667,11 +1708,11 @@
       <c r="D16" s="10">
         <v>8</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>3</v>
       </c>
@@ -1682,11 +1723,11 @@
       <c r="D17" s="10">
         <v>8</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
         <v>13</v>
       </c>
@@ -1697,11 +1738,11 @@
       <c r="D18" s="10">
         <v>8</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="10" t="s">
         <v>14</v>
       </c>
@@ -1712,11 +1753,11 @@
       <c r="D19" s="10">
         <v>20</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="58">
         <v>1500</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>15</v>
       </c>
@@ -1727,11 +1768,11 @@
       <c r="D20" s="10">
         <v>8</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>8</v>
       </c>
@@ -1742,11 +1783,11 @@
       <c r="D21" s="10">
         <v>8</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>16</v>
       </c>
@@ -1756,12 +1797,18 @@
         <f>SUM(D23:D29)</f>
         <v>160</v>
       </c>
-      <c r="E22" s="9">
+      <c r="E22" s="57">
         <f>SUM(E23:E29)</f>
         <v>12000</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="59">
+        <v>75</v>
+      </c>
+      <c r="G22" s="60" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
         <v>17</v>
       </c>
@@ -1772,11 +1819,11 @@
       <c r="D23" s="10">
         <v>80</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="58">
         <v>6000</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>18</v>
       </c>
@@ -1787,11 +1834,11 @@
       <c r="D24" s="10">
         <v>16</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="58">
         <v>1200</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>19</v>
       </c>
@@ -1802,11 +1849,11 @@
       <c r="D25" s="10">
         <v>16</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="58">
         <v>1200</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="10" t="s">
         <v>3</v>
       </c>
@@ -1817,11 +1864,11 @@
       <c r="D26" s="10">
         <v>8</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>15</v>
       </c>
@@ -1832,11 +1879,11 @@
       <c r="D27" s="10">
         <v>8</v>
       </c>
-      <c r="E27" s="10">
+      <c r="E27" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>4</v>
       </c>
@@ -1847,11 +1894,11 @@
       <c r="D28" s="10">
         <v>8</v>
       </c>
-      <c r="E28" s="10">
+      <c r="E28" s="58">
         <v>600</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>20</v>
       </c>
@@ -1862,11 +1909,11 @@
       <c r="D29" s="10">
         <v>24</v>
       </c>
-      <c r="E29" s="10">
+      <c r="E29" s="58">
         <v>1800</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>21</v>
       </c>
@@ -1876,12 +1923,18 @@
         <f>SUM(D31:D48)</f>
         <v>304</v>
       </c>
-      <c r="E30" s="9">
+      <c r="E30" s="57">
         <f>SUM(E31:E48)</f>
         <v>28880</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="59">
+        <v>95</v>
+      </c>
+      <c r="G30" s="60" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>19</v>
       </c>
@@ -1892,11 +1945,11 @@
       <c r="D31" s="10">
         <v>16</v>
       </c>
-      <c r="E31" s="10">
+      <c r="E31" s="58">
         <v>1520</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="10" t="s">
         <v>22</v>
       </c>
@@ -1907,7 +1960,7 @@
       <c r="D32" s="10">
         <v>16</v>
       </c>
-      <c r="E32" s="10">
+      <c r="E32" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -1922,7 +1975,7 @@
       <c r="D33" s="10">
         <v>8</v>
       </c>
-      <c r="E33" s="10">
+      <c r="E33" s="58">
         <v>760</v>
       </c>
     </row>
@@ -1937,7 +1990,7 @@
       <c r="D34" s="10">
         <v>16</v>
       </c>
-      <c r="E34" s="10">
+      <c r="E34" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -1952,7 +2005,7 @@
       <c r="D35" s="10">
         <v>16</v>
       </c>
-      <c r="E35" s="10">
+      <c r="E35" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -1967,7 +2020,7 @@
       <c r="D36" s="10">
         <v>16</v>
       </c>
-      <c r="E36" s="10">
+      <c r="E36" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -1982,7 +2035,7 @@
       <c r="D37" s="10">
         <v>16</v>
       </c>
-      <c r="E37" s="10">
+      <c r="E37" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -1997,7 +2050,7 @@
       <c r="D38" s="10">
         <v>24</v>
       </c>
-      <c r="E38" s="10">
+      <c r="E38" s="58">
         <v>2280</v>
       </c>
     </row>
@@ -2012,7 +2065,7 @@
       <c r="D39" s="10">
         <v>16</v>
       </c>
-      <c r="E39" s="10">
+      <c r="E39" s="58">
         <v>1520</v>
       </c>
     </row>
@@ -2027,7 +2080,7 @@
       <c r="D40" s="10">
         <v>8</v>
       </c>
-      <c r="E40" s="10">
+      <c r="E40" s="58">
         <v>760</v>
       </c>
     </row>
@@ -2042,7 +2095,7 @@
       <c r="D41" s="10">
         <v>40</v>
       </c>
-      <c r="E41" s="10">
+      <c r="E41" s="58">
         <v>3800</v>
       </c>
     </row>
@@ -2057,7 +2110,7 @@
       <c r="D42" s="10">
         <v>8</v>
       </c>
-      <c r="E42" s="10">
+      <c r="E42" s="58">
         <v>760</v>
       </c>
     </row>
@@ -2072,7 +2125,7 @@
       <c r="D43" s="10">
         <v>8</v>
       </c>
-      <c r="E43" s="10">
+      <c r="E43" s="58">
         <v>760</v>
       </c>
     </row>
@@ -2087,7 +2140,7 @@
       <c r="D44" s="10">
         <v>8</v>
       </c>
-      <c r="E44" s="10">
+      <c r="E44" s="58">
         <v>760</v>
       </c>
     </row>
@@ -2102,7 +2155,7 @@
       <c r="D45" s="10">
         <v>40</v>
       </c>
-      <c r="E45" s="10">
+      <c r="E45" s="58">
         <v>3800</v>
       </c>
     </row>
@@ -2117,7 +2170,7 @@
       <c r="D46" s="10">
         <v>24</v>
       </c>
-      <c r="E46" s="10">
+      <c r="E46" s="58">
         <v>2280</v>
       </c>
     </row>
@@ -2132,7 +2185,7 @@
       <c r="D47" s="10">
         <v>8</v>
       </c>
-      <c r="E47" s="10">
+      <c r="E47" s="58">
         <v>760</v>
       </c>
     </row>
@@ -2147,11 +2200,11 @@
       <c r="D48" s="10">
         <v>16</v>
       </c>
-      <c r="E48" s="10">
+      <c r="E48" s="58">
         <v>1520</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>31</v>
       </c>
@@ -2161,12 +2214,18 @@
         <f>SUM(D50:D55)</f>
         <v>80</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="57">
         <f>SUM(E50:E55)</f>
         <v>5200</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="59">
+        <v>65</v>
+      </c>
+      <c r="G49" s="60" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
         <v>3</v>
       </c>
@@ -2177,11 +2236,11 @@
       <c r="D50" s="10">
         <v>8</v>
       </c>
-      <c r="E50" s="10">
+      <c r="E50" s="58">
         <v>520</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
         <v>6</v>
       </c>
@@ -2192,11 +2251,11 @@
       <c r="D51" s="10">
         <v>8</v>
       </c>
-      <c r="E51" s="10">
+      <c r="E51" s="58">
         <v>520</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
         <v>32</v>
       </c>
@@ -2207,11 +2266,11 @@
       <c r="D52" s="10">
         <v>40</v>
       </c>
-      <c r="E52" s="10">
+      <c r="E52" s="58">
         <v>2600</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
         <v>24</v>
       </c>
@@ -2222,11 +2281,11 @@
       <c r="D53" s="10">
         <v>16</v>
       </c>
-      <c r="E53" s="10">
+      <c r="E53" s="58">
         <v>1040</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
         <v>7</v>
       </c>
@@ -2237,11 +2296,11 @@
       <c r="D54" s="10">
         <v>4</v>
       </c>
-      <c r="E54" s="10">
+      <c r="E54" s="58">
         <v>260</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>4</v>
       </c>
@@ -2252,11 +2311,11 @@
       <c r="D55" s="10">
         <v>4</v>
       </c>
-      <c r="E55" s="10">
+      <c r="E55" s="58">
         <v>260</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
         <v>33</v>
       </c>
@@ -2265,12 +2324,12 @@
       <c r="D56" s="8">
         <v>0</v>
       </c>
-      <c r="E56" s="8">
+      <c r="E56" s="56">
         <f>SUM(E73,E71,E69,E67,E65,E63,E61,E59,E57)</f>
         <v>104700</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
         <v>23</v>
       </c>
@@ -2279,12 +2338,18 @@
       <c r="D57" s="9">
         <v>0</v>
       </c>
-      <c r="E57" s="9">
+      <c r="E57" s="57">
         <f>SUM(E58)</f>
         <v>20000</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F57" s="59">
+        <v>20000</v>
+      </c>
+      <c r="G57" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="10" t="s">
         <v>23</v>
       </c>
@@ -2297,11 +2362,11 @@
       <c r="D58" s="10">
         <v>0</v>
       </c>
-      <c r="E58" s="10">
+      <c r="E58" s="58">
         <v>20000</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>34</v>
       </c>
@@ -2310,12 +2375,18 @@
       <c r="D59" s="9">
         <v>0</v>
       </c>
-      <c r="E59" s="9">
+      <c r="E59" s="57">
         <f>SUM(E60)</f>
         <v>15000</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F59" s="59">
+        <v>15000</v>
+      </c>
+      <c r="G59" s="60" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="10" t="s">
         <v>6</v>
       </c>
@@ -2328,11 +2399,11 @@
       <c r="D60" s="10">
         <v>0</v>
       </c>
-      <c r="E60" s="10">
+      <c r="E60" s="58">
         <v>15000</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>35</v>
       </c>
@@ -2341,12 +2412,18 @@
       <c r="D61" s="9">
         <v>0</v>
       </c>
-      <c r="E61" s="9">
+      <c r="E61" s="57">
         <f>SUM(E62)</f>
         <v>500</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F61" s="59">
+        <v>500</v>
+      </c>
+      <c r="G61" s="60" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="10" t="s">
         <v>6</v>
       </c>
@@ -2359,11 +2436,11 @@
       <c r="D62" s="10">
         <v>0</v>
       </c>
-      <c r="E62" s="10">
+      <c r="E62" s="58">
         <v>500</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
         <v>36</v>
       </c>
@@ -2372,12 +2449,18 @@
       <c r="D63" s="9">
         <v>0</v>
       </c>
-      <c r="E63" s="9">
+      <c r="E63" s="57">
         <f>SUM(E64)</f>
         <v>12000</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F63" s="59">
+        <v>12000</v>
+      </c>
+      <c r="G63" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="10" t="s">
         <v>23</v>
       </c>
@@ -2390,11 +2473,11 @@
       <c r="D64" s="10">
         <v>0</v>
       </c>
-      <c r="E64" s="10">
+      <c r="E64" s="58">
         <v>12000</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
         <v>37</v>
       </c>
@@ -2403,12 +2486,18 @@
       <c r="D65" s="9">
         <v>0</v>
       </c>
-      <c r="E65" s="9">
+      <c r="E65" s="57">
         <f>SUM(E66)</f>
         <v>3200</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F65" s="59">
+        <v>800</v>
+      </c>
+      <c r="G65" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="10" t="s">
         <v>6</v>
       </c>
@@ -2416,16 +2505,16 @@
         <v>37</v>
       </c>
       <c r="C66" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D66" s="10">
         <v>0</v>
       </c>
-      <c r="E66" s="10">
+      <c r="E66" s="58">
         <v>3200</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>38</v>
       </c>
@@ -2434,12 +2523,18 @@
       <c r="D67" s="9">
         <v>0</v>
       </c>
-      <c r="E67" s="9">
+      <c r="E67" s="57">
         <f>SUM(E68)</f>
         <v>24000</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F67" s="59">
+        <v>6000</v>
+      </c>
+      <c r="G67" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="10" t="s">
         <v>6</v>
       </c>
@@ -2447,16 +2542,16 @@
         <v>38</v>
       </c>
       <c r="C68" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D68" s="10">
         <v>0</v>
       </c>
-      <c r="E68" s="10">
+      <c r="E68" s="58">
         <v>24000</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
         <v>39</v>
       </c>
@@ -2465,12 +2560,18 @@
       <c r="D69" s="9">
         <v>0</v>
       </c>
-      <c r="E69" s="9">
+      <c r="E69" s="57">
         <f>SUM(E70)</f>
         <v>10000</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F69" s="59">
+        <v>10000</v>
+      </c>
+      <c r="G69" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="10" t="s">
         <v>5</v>
       </c>
@@ -2483,11 +2584,11 @@
       <c r="D70" s="10">
         <v>0</v>
       </c>
-      <c r="E70" s="10">
+      <c r="E70" s="58">
         <v>10000</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
         <v>40</v>
       </c>
@@ -2496,12 +2597,18 @@
       <c r="D71" s="9">
         <v>0</v>
       </c>
-      <c r="E71" s="9">
+      <c r="E71" s="57">
         <f>SUM(E72)</f>
         <v>15000</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F71" s="59">
+        <v>15000</v>
+      </c>
+      <c r="G71" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="10" t="s">
         <v>24</v>
       </c>
@@ -2514,11 +2621,11 @@
       <c r="D72" s="10">
         <v>0</v>
       </c>
-      <c r="E72" s="10">
+      <c r="E72" s="58">
         <v>15000</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="s">
         <v>41</v>
       </c>
@@ -2527,12 +2634,18 @@
       <c r="D73" s="9">
         <v>0</v>
       </c>
-      <c r="E73" s="9">
+      <c r="E73" s="57">
         <f>SUM(E74)</f>
         <v>5000</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F73" s="59">
+        <v>5000</v>
+      </c>
+      <c r="G73" s="60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>6</v>
       </c>
@@ -2545,17 +2658,17 @@
       <c r="D74" s="10">
         <v>0</v>
       </c>
-      <c r="E74" s="10">
+      <c r="E74" s="58">
         <v>5000</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="52" t="s">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="49" t="s">
         <v>159</v>
       </c>
-      <c r="B76" s="52"/>
-      <c r="C76" s="52"/>
-      <c r="D76" s="52"/>
+      <c r="B76" s="49"/>
+      <c r="C76" s="49"/>
+      <c r="D76" s="49"/>
       <c r="E76" s="29">
         <f>SUM(E2,E56)</f>
         <v>170340</v>
@@ -3778,10 +3891,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="52" t="s">
         <v>179</v>
       </c>
-      <c r="B9" s="54"/>
+      <c r="B9" s="52"/>
       <c r="C9" s="21">
         <f>0.91+(0.01*C8)</f>
         <v>1.0499000000000001</v>
@@ -3861,10 +3974,10 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="52" t="s">
         <v>199</v>
       </c>
-      <c r="B18" s="54"/>
+      <c r="B18" s="52"/>
       <c r="C18" s="21">
         <f>C13*C14*C15*C16*C17</f>
         <v>0.72897300000000009</v>
@@ -4056,13 +4169,13 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="54" t="s">
+      <c r="A7" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="B7" s="54"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
+      <c r="B7" s="52"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
       <c r="F7" s="21">
         <f>SUM(F2:F6)</f>
         <v>115</v>
@@ -4075,13 +4188,13 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="53" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="55"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
       <c r="F8" s="7">
         <f>F7*I18</f>
         <v>134.54999999999998</v>
@@ -4195,23 +4308,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="54" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
       <c r="E1" s="30">
         <v>0.08</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="55" t="s">
         <v>209</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
       <c r="E2" s="31" t="s">
         <v>159</v>
       </c>
@@ -4402,12 +4515,12 @@
       <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="54" t="s">
         <v>217</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
       <c r="E15" s="38">
         <f>(E10/E6)-1</f>
         <v>23.373525319366614</v>

</xml_diff>